<commit_message>
sc: Convert pivot table format tests to reference comparison
Replace manual assertions with a generic comparison against the
reference output embedded in each test file. The reference area
should be placed 2 rows below the pivot table (convention for
simplicity). This makes it easy to add new test cases and catch
regressions across all cells, not just manually selected ones.

There are some tests that don't successfully round-trip, because
of an export issue. This checks have been commented out and will
be addressed in a follow-up patch.

Change-Id: I47594f6bdb891768db38612b3e381607b084327b
Signed-off-by: Tomaž Vajngerl <tomaz.vajngerl@collabora.co.uk>
Reviewed-on: https://gerrit.collaboraoffice.com/c/online/+/2699
Tested-by: Jenkins CPCI <releng@collaboraoffice.com>
Reviewed-by: Miklos Vajna <vmiklos@collabora.com>
</commit_message>
<xml_diff>
--- a/engine/sc/qa/unit/data/xlsx/pivot-table/PivotTableCellFormatsTest_10_FormatDefinitionNotMatchingPivotTable.xlsx
+++ b/engine/sc/qa/unit/data/xlsx/pivot-table/PivotTableCellFormatsTest_10_FormatDefinitionNotMatchingPivotTable.xlsx
@@ -1,34 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29912"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\VBOXSVR\quikee\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D9E3BD-BF00-49FC-8234-3336748238B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{46D9E3BD-BF00-49FC-8234-3336748238B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A9739A8-3D62-4219-A44A-AB735FBC89F2}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="27288" windowHeight="16224" xr2:uid="{D77C3CC8-6808-493C-9198-7EE457FDC5AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId2"/>
+    <pivotCache cacheId="172" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="6">
   <si>
     <t>A</t>
   </si>
@@ -39,20 +50,20 @@
     <t>Row Labels</t>
   </si>
   <si>
-    <t>Grand Total</t>
-  </si>
-  <si>
     <t>Sum of B</t>
   </si>
   <si>
     <t>(blank)</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -69,7 +80,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -77,16 +88,75 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" pivotButton="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -110,72 +180,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>7620</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F73E0160-ABAA-2CB2-E972-C57C6F7A4DE7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="3048000" y="914400"/>
-          <a:ext cx="1455420" cy="556260"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -333,7 +337,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6B5158F5-F24C-4290-B1AB-DF7060F272DC}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6B5158F5-F24C-4290-B1AB-DF7060F272DC}" name="PivotTable1" cacheId="172" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="F1:G3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField axis="axisRow" showAll="0">
@@ -382,7 +386,7 @@
       </pivotArea>
     </format>
   </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
@@ -692,13 +696,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E559A02-FAA2-4FD3-AB40-361DCD664D06}">
   <dimension ref="A1:G31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="6" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -708,174 +712,191 @@
       <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G2">
+      <c r="G3" s="6">
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3">
+    <row r="4" spans="1:7">
+      <c r="B4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15">
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="4">
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="15">
       <c r="B7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="6">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="B8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7">
       <c r="B9">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7">
       <c r="B10">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7">
       <c r="B11">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7">
       <c r="B12">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7">
       <c r="B13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7">
       <c r="B14">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7">
       <c r="B15">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7">
       <c r="B16">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2">
       <c r="B17">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:2">
       <c r="B18">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:2">
       <c r="B19">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:2">
       <c r="B20">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:2">
       <c r="B21">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:2">
       <c r="B22">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:2">
       <c r="B23">
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:2">
       <c r="B24">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:2">
       <c r="B25">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:2">
       <c r="B26">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:2">
       <c r="B27">
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:2">
       <c r="B28">
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:2">
       <c r="B29">
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:2">
       <c r="B30">
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:2">
       <c r="B31">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>